<commit_message>
Polling bias slider, Fundamentals rename, poll sparkline, undecided share, tooltip trend lines
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Districts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mail-In" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Senate" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Polls" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0;-0.0"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +58,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -93,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -104,6 +109,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -469,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -557,7 +564,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10870,4 +10876,1173 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Pollster</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Start date</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>End date</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Dem %</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Rep %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>46300</v>
+      </c>
+      <c r="D2" t="n">
+        <v>51</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>46300</v>
+      </c>
+      <c r="D3" t="n">
+        <v>44</v>
+      </c>
+      <c r="E3" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>46299</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pew Research</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>46299</v>
+      </c>
+      <c r="D5" t="n">
+        <v>44</v>
+      </c>
+      <c r="E5" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cygnal</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D6" t="n">
+        <v>52</v>
+      </c>
+      <c r="E6" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CBS News</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D7" t="n">
+        <v>54</v>
+      </c>
+      <c r="E7" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Harvard-Harris</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="D8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E8" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="D9" t="n">
+        <v>53</v>
+      </c>
+      <c r="E9" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="D10" t="n">
+        <v>47</v>
+      </c>
+      <c r="E10" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Quinnipiac</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="D11" t="n">
+        <v>51</v>
+      </c>
+      <c r="E11" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="D12" t="n">
+        <v>50</v>
+      </c>
+      <c r="E12" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="D13" t="n">
+        <v>48</v>
+      </c>
+      <c r="E13" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Emerson</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="D14" t="n">
+        <v>53</v>
+      </c>
+      <c r="E14" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="D15" t="n">
+        <v>52</v>
+      </c>
+      <c r="E15" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Echelon Insights</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="D16" t="n">
+        <v>51</v>
+      </c>
+      <c r="E16" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Wall Street Journal</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="D17" t="n">
+        <v>50</v>
+      </c>
+      <c r="E17" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D18" t="n">
+        <v>50</v>
+      </c>
+      <c r="E18" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D19" t="n">
+        <v>43</v>
+      </c>
+      <c r="E19" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Quantus Insights</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="D20" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="D21" t="n">
+        <v>49</v>
+      </c>
+      <c r="E21" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D22" t="n">
+        <v>49</v>
+      </c>
+      <c r="E22" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NPR/PBS/Marist</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="D23" t="n">
+        <v>53</v>
+      </c>
+      <c r="E23" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Big Data Poll</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="D24" t="n">
+        <v>51</v>
+      </c>
+      <c r="E24" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NBC News</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="D25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RMG Research</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="D26" t="n">
+        <v>52</v>
+      </c>
+      <c r="E26" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>FOX News</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="D27" t="n">
+        <v>51</v>
+      </c>
+      <c r="E27" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="D28" t="n">
+        <v>51</v>
+      </c>
+      <c r="E28" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C29" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="D29" t="n">
+        <v>44</v>
+      </c>
+      <c r="E29" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="D30" t="n">
+        <v>49</v>
+      </c>
+      <c r="E30" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NY Times/Siena</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CBS News</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>46276</v>
+      </c>
+      <c r="D32" t="n">
+        <v>54</v>
+      </c>
+      <c r="E32" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>46274</v>
+      </c>
+      <c r="D33" t="n">
+        <v>47</v>
+      </c>
+      <c r="E33" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Marquette</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n">
+        <v>46267</v>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>46274</v>
+      </c>
+      <c r="D34" t="n">
+        <v>54</v>
+      </c>
+      <c r="E34" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="n">
+        <v>46269</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>46273</v>
+      </c>
+      <c r="D35" t="n">
+        <v>49</v>
+      </c>
+      <c r="E35" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Quinnipiac</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>46271</v>
+      </c>
+      <c r="D36" t="n">
+        <v>49</v>
+      </c>
+      <c r="E36" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>46271</v>
+      </c>
+      <c r="D37" t="n">
+        <v>46</v>
+      </c>
+      <c r="E37" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cygnal</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>46266</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>46267</v>
+      </c>
+      <c r="D38" t="n">
+        <v>51</v>
+      </c>
+      <c r="E38" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Financial Times</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>46267</v>
+      </c>
+      <c r="D39" t="n">
+        <v>52</v>
+      </c>
+      <c r="E39" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D40" t="n">
+        <v>46</v>
+      </c>
+      <c r="E40" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D41" t="n">
+        <v>43</v>
+      </c>
+      <c r="E41" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D42" t="n">
+        <v>47</v>
+      </c>
+      <c r="E42" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Harvard-Harris</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D43" t="n">
+        <v>49</v>
+      </c>
+      <c r="E43" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Quantus Insights</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="n">
+        <v>46260</v>
+      </c>
+      <c r="C44" s="11" t="n">
+        <v>46262</v>
+      </c>
+      <c r="D44" t="n">
+        <v>50</v>
+      </c>
+      <c r="E44" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="n">
+        <v>46257</v>
+      </c>
+      <c r="C45" s="11" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D45" t="n">
+        <v>41</v>
+      </c>
+      <c r="E45" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D46" t="n">
+        <v>46</v>
+      </c>
+      <c r="E46" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D47" t="n">
+        <v>41</v>
+      </c>
+      <c r="E47" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Emerson</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D48" t="n">
+        <v>51</v>
+      </c>
+      <c r="E48" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D49" t="n">
+        <v>46</v>
+      </c>
+      <c r="E49" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D50" t="n">
+        <v>41</v>
+      </c>
+      <c r="E50" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Echelon Insights</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D51" t="n">
+        <v>50</v>
+      </c>
+      <c r="E51" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="n">
+        <v>46244</v>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D52" t="n">
+        <v>46</v>
+      </c>
+      <c r="E52" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Financial Times</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D53" t="n">
+        <v>51</v>
+      </c>
+      <c r="E53" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D54" t="n">
+        <v>46</v>
+      </c>
+      <c r="E54" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Cygnal</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>46241</v>
+      </c>
+      <c r="D55" t="n">
+        <v>49</v>
+      </c>
+      <c r="E55" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Quantus Insights</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D56" t="n">
+        <v>49</v>
+      </c>
+      <c r="E56" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>RMG Research</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="n">
+        <v>46231</v>
+      </c>
+      <c r="C57" s="11" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D57" t="n">
+        <v>47</v>
+      </c>
+      <c r="E57" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D58" t="n">
+        <v>46</v>
+      </c>
+      <c r="E58" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="n">
+        <v>46232</v>
+      </c>
+      <c r="C59" s="11" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D59" t="n">
+        <v>42</v>
+      </c>
+      <c r="E59" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D60" t="n">
+        <v>46</v>
+      </c>
+      <c r="E60" t="n">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update polling data: generic ballot to D+7.9 (Oct 11, 2026)
- Generic-ballot input refreshed from aggregators (RealClearPolitics
  D+7.9; FiftyPlusOne D+8.0, Oct 10) down from D+8.9; source and
  "data updated" stamp updated
- Rebuilt data.js and 2026-house-forecast.html via update_forecast.py;
  opening tally now D 232 / R 203
- Individual polls unchanged (no new generic-ballot polls past Oct 5)
- Refreshed link-preview card (assets/og-image.png) to 232/203

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -497,6 +497,11 @@
           <t>Edit the blue cells, save, then load this file on the page (or run update_forecast.py).</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>October 11, 2026</t>
+        </is>
+      </c>
     </row>
     <row r="3"/>
     <row r="4">
@@ -523,7 +528,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -539,7 +544,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Nate Silver · Silver Bulletin (Oct. 8, 2026)</t>
+          <t>RealClearPolitics average (Oct. 10, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -556,7 +561,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 9, 2026</t>
+          <t>October 11, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update polling data (Oct 16, 2026): +11 polls, generic ballot D+8.0
- Added 11 new generic-ballot polls with field dates Oct 6-13
  (FOX, Economist/YouGov, RMG, Morning Consult, AP/NORC, Cygnal,
  NewsNation, Center Square/NPI, Financial Times, Rasmussen, THP/MM)
  -> Polls sheet now 90 entries
- Generic ballot to D+8.0 (RealClearPolitics average, Oct 16);
  "data updated" stamp refreshed
- Rebuilt data.js and 2026-house-forecast.html; opening tally
  unchanged at D 232 / R 203

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0;-0.0"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -98,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,6 +112,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>October 11, 2026</t>
+          <t>October 16, 2026</t>
         </is>
       </c>
     </row>
@@ -528,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -544,7 +546,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>RealClearPolitics average (Oct. 10, 2026)</t>
+          <t>RealClearPolitics average (Oct. 16, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -561,7 +563,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 11, 2026</t>
+          <t>October 16, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -10890,7 +10892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12428,6 +12430,215 @@
         <v>49</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>FOX News</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C81" s="12" t="n">
+        <v>46307</v>
+      </c>
+      <c r="D81" t="n">
+        <v>54</v>
+      </c>
+      <c r="E81" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C82" s="12" t="n">
+        <v>46307</v>
+      </c>
+      <c r="D82" t="n">
+        <v>49</v>
+      </c>
+      <c r="E82" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>RMG Research</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C83" s="12" t="n">
+        <v>46308</v>
+      </c>
+      <c r="D83" t="n">
+        <v>54</v>
+      </c>
+      <c r="E83" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C84" s="12" t="n">
+        <v>46306</v>
+      </c>
+      <c r="D84" t="n">
+        <v>50</v>
+      </c>
+      <c r="E84" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>AP/NORC</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C85" s="12" t="n">
+        <v>46307</v>
+      </c>
+      <c r="D85" t="n">
+        <v>47</v>
+      </c>
+      <c r="E85" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Cygnal</t>
+        </is>
+      </c>
+      <c r="B86" s="12" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C86" s="12" t="n">
+        <v>46305</v>
+      </c>
+      <c r="D86" t="n">
+        <v>51</v>
+      </c>
+      <c r="E86" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>NewsNation</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C87" s="12" t="n">
+        <v>46304</v>
+      </c>
+      <c r="D87" t="n">
+        <v>49</v>
+      </c>
+      <c r="E87" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Center Square/NPI</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C88" s="12" t="n">
+        <v>46302</v>
+      </c>
+      <c r="D88" t="n">
+        <v>47</v>
+      </c>
+      <c r="E88" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Financial Times</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="n">
+        <v>46298</v>
+      </c>
+      <c r="C89" s="12" t="n">
+        <v>46301</v>
+      </c>
+      <c r="D89" t="n">
+        <v>52</v>
+      </c>
+      <c r="E89" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C90" s="12" t="n">
+        <v>46302</v>
+      </c>
+      <c r="D90" t="n">
+        <v>49</v>
+      </c>
+      <c r="E90" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>THP/MM</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C91" s="12" t="n">
+        <v>46301</v>
+      </c>
+      <c r="D91" t="n">
+        <v>54</v>
+      </c>
+      <c r="E91" t="n">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update polling data (Oct 18, 2026): generic ballot D+8.2
- Generic ballot to D+8.2 (RealClearPolitics average, Oct 18);
  average ticked up from D+8.0 (FiftyPlusOne has D+9)
- No new individual polls: latest fieldwork still ends Oct 13
- Rebuilt data.js and 2026-house-forecast.html; opening tally
  now D 233 / R 202 (one seat flips D)
- Refreshed link-preview card (assets/og-image.png) to 233/202

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>October 16, 2026</t>
+          <t>October 18, 2026</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>RealClearPolitics average (Oct. 16, 2026)</t>
+          <t>RealClearPolitics average (Oct. 18, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 16, 2026</t>
+          <t>October 18, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update polling data (Oct 20, 2026): +3 polls, generic ballot D+8.6
- Added 3 new generic-ballot polls (Reuters/Ipsos 10/16-19,
  Morning Consult 10/12-18, Rasmussen 10/8-14) -> Polls sheet now 93
- Generic ballot to D+8.6 (RealClearPolitics average, Oct 20),
  up from D+8.2 (FiftyPlusOne has D+9)
- Rebuilt data.js and 2026-house-forecast.html; opening tally
  now D 235 / R 200
- Refreshed link-preview card (assets/og-image.png) to 235/200

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>October 18, 2026</t>
+          <t>October 20, 2026</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>RealClearPolitics average (Oct. 18, 2026)</t>
+          <t>RealClearPolitics average (Oct. 20, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 18, 2026</t>
+          <t>October 20, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -10892,7 +10892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12639,6 +12639,63 @@
         <v>42</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Reuters/Ipsos</t>
+        </is>
+      </c>
+      <c r="B92" s="12" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C92" s="12" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D92" t="n">
+        <v>47</v>
+      </c>
+      <c r="E92" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C93" s="12" t="n">
+        <v>46313</v>
+      </c>
+      <c r="D93" t="n">
+        <v>50</v>
+      </c>
+      <c r="E93" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Rasmussen Reports</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C94" s="12" t="n">
+        <v>46309</v>
+      </c>
+      <c r="D94" t="n">
+        <v>48</v>
+      </c>
+      <c r="E94" t="n">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update House + Senate from multiple sources, triple-verified (Oct 21, 2026)
House:
- Generic ballot to D+8.2 (consensus of RCP 8.3, Silver Bulletin 8.9,
  DDHQ 7.5, FiftyPlusOne 8.0); added Echelon Insights poll (10/15-19)
  -> Polls sheet now 94; House tally D 233 / R 202

Senate (per-race Dem win %, blend of Silver Bulletin + DDHQ, tempered by
Cook/Sabato/Inside Elections consensus):
- Democrats now favored to flip: projected 52 D / 48 R (was R-held)
- Flips: NC, AK, TX, ME, OH; big shifts NC 83->90, OH 51->63, ME 53->64,
  KS 35->44, TX 57->52, GA 88->92
- Updated Senate sheet, data.js meta.senate, and the source note
- Refreshed link-preview card to 233/202

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>October 20, 2026</t>
+          <t>October 21, 2026</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>RealClearPolitics average (Oct. 20, 2026)</t>
+          <t>Avg of RCP, Silver Bulletin, DDHQ, 50+1 (Oct. 21, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 20, 2026</t>
+          <t>October 21, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -10115,10 +10115,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Per-race Democratic win probability (%). 34 Democratic-held seats are not up; 51 needed for control. Decision Desk HQ / The Hill forecast, Oct. 9, 2026.</t>
-        </is>
-      </c>
-    </row>
+          <t>Per-race Democratic win probability (%). Blend of Silver Bulletin, Decision Desk HQ, and Cook/Sabato/Inside Elections consensus, Oct. 21, 2026. 34 Democratic-held seats not up; 51 needed for control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10153,7 +10154,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -10195,7 +10196,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
@@ -10237,7 +10238,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -10258,7 +10259,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
@@ -10321,7 +10322,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
@@ -10342,7 +10343,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
@@ -10363,7 +10364,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
@@ -10384,7 +10385,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -10405,11 +10406,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Lean D</t>
+          <t>Likely D</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -10426,7 +10427,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
@@ -10447,11 +10448,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Toss-Up (flip)</t>
+          <t>Lean D (flip)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -10468,7 +10469,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
@@ -10489,11 +10490,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Toss-Up (flip)</t>
+          <t>Lean D (flip)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -10510,7 +10511,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
@@ -10531,7 +10532,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
@@ -10552,11 +10553,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-Up</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -10573,7 +10574,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
@@ -10594,11 +10595,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -10657,7 +10658,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
@@ -10720,7 +10721,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
@@ -10741,11 +10742,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Likely R</t>
+          <t>Safe R</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -10762,7 +10763,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
@@ -10892,7 +10893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12696,6 +12697,25 @@
         <v>44</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Echelon Insights</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C95" s="12" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D95" t="n">
+        <v>50</v>
+      </c>
+      <c r="E95" t="n">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update polling data (Oct 24, 2026): generic ballot D+8.5, +1 poll
- Generic ballot to D+8.5, consensus of RCP 8.1, Silver Bulletin 9.1,
  DDHQ 7.9, FiftyPlusOne 9.0 (up from D+8.2)
- Added Economist/YouGov (10/19-20) -> Polls sheet now 95
- Rebuilt data.js and 2026-house-forecast.html; House tally
  D 235 / R 200; Senate unchanged at 52 D / 48 R
- Refreshed link-preview card to 235/200

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>October 21, 2026</t>
+          <t>October 24, 2026</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Avg of RCP, Silver Bulletin, DDHQ, 50+1 (Oct. 21, 2026)</t>
+          <t>Avg of RCP, Silver Bulletin, DDHQ, 50+1 (Oct. 24, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 21, 2026</t>
+          <t>October 24, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -10119,7 +10119,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10893,7 +10892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12716,6 +12715,25 @@
         <v>45</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Economist/YouGov</t>
+        </is>
+      </c>
+      <c r="B96" s="12" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C96" s="12" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D96" t="n">
+        <v>50</v>
+      </c>
+      <c r="E96" t="n">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update polling data (Oct 26, 2026): generic ballot D+8.6, +1 poll
- Generic ballot to D+8.6, consensus of RCP 8.3, Silver Bulletin 9.1,
  DDHQ 8.1, FiftyPlusOne 9.0 (up from D+8.5)
- Added CBS News (10/21-23) -> Polls sheet now 96
- Rebuilt data.js and 2026-house-forecast.html; tallies unchanged
  (House D 235 / R 200, Senate 52 D / 48 R)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>October 24, 2026</t>
+          <t>October 26, 2026</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Avg of RCP, Silver Bulletin, DDHQ, 50+1 (Oct. 24, 2026)</t>
+          <t>Avg of RCP, Silver Bulletin, DDHQ, 50+1 (Oct. 26, 2026)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>October 24, 2026</t>
+          <t>October 26, 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -10892,7 +10892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12734,6 +12734,25 @@
         <v>43</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CBS News</t>
+        </is>
+      </c>
+      <c r="B97" s="12" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C97" s="12" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D97" t="n">
+        <v>53</v>
+      </c>
+      <c r="E97" t="n">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tooltips: per-race trend sparkline from the polling average; add Morning Consult 10/19-25 (104 polls)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZRYyi6ihXen8gdMRgfCfh
</commit_message>
<xml_diff>
--- a/house-polling.xlsx
+++ b/house-polling.xlsx
@@ -507,6 +507,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10893,7 +10894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12885,6 +12886,25 @@
       </c>
       <c r="E104" t="n">
         <v>42</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Morning Consult</t>
+        </is>
+      </c>
+      <c r="B105" s="12" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C105" s="12" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D105" t="n">
+        <v>50</v>
+      </c>
+      <c r="E105" t="n">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>